<commit_message>
docs(xlsx): actualizar esquema con Frontend Mobile + Errores ERR-01..22 (sesión 19abr)
</commit_message>
<xml_diff>
--- a/ESQUEMA_SISTEMA_PORRA2026.xlsx
+++ b/ESQUEMA_SISTEMA_PORRA2026.xlsx
@@ -1,17 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Edge Functions" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Actor Apify + pg_cron" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="APIs + DB" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Flujo + Leyenda" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IDs SofaScore + Costes" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Edge Functions" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Actor Apify + pg_cron" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="APIs + DB" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Flujo + Leyenda" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="IDs SofaScore + Costes" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Frontend Mobile" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Errores ERR-01..ERR-22" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -21,7 +23,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -62,8 +64,19 @@
       <color rgb="001F3864"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <sz val="12"/>
+    </font>
   </fonts>
-  <fills count="12">
+  <fills count="14">
     <fill>
       <patternFill/>
     </fill>
@@ -120,8 +133,18 @@
         <fgColor rgb="00FCE4D6"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F4E78"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9E1F2"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -143,11 +166,55 @@
         <color rgb="00BFBFBF"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -244,6 +311,21 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="13" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -610,7 +692,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -626,6 +708,10 @@
           <t>PORRA MUNDIAL 2026 — Edge Functions Supabase (cmyfyswystjgzdwbqyyb)</t>
         </is>
       </c>
+      <c r="B1" s="33" t="n"/>
+      <c r="C1" s="33" t="n"/>
+      <c r="D1" s="33" t="n"/>
+      <c r="E1" s="34" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -657,7 +743,7 @@
     <row r="3" ht="55" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>porra-match-live v12</t>
+          <t>porra-match-live v13</t>
         </is>
       </c>
       <c r="B3" s="4" t="inlineStr">
@@ -684,7 +770,7 @@
     <row r="4" ht="55" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>porra-apify-webhook v5</t>
+          <t>porra-apify-webhook v7</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
@@ -792,7 +878,7 @@
     <row r="8" ht="55" customHeight="1">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>update-results v2</t>
+          <t>update-results v4</t>
         </is>
       </c>
       <c r="B8" s="7" t="inlineStr">
@@ -873,7 +959,7 @@
     <row r="11" ht="55" customHeight="1">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>porra-fix-encoding v4</t>
+          <t>porra-fix-encoding v6</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
@@ -948,6 +1034,33 @@
       <c r="E13" s="11" t="inlineStr">
         <is>
           <t>❌ Placeholder</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="35" t="inlineStr">
+        <is>
+          <t>create-league v2</t>
+        </is>
+      </c>
+      <c r="B14" s="35" t="inlineStr">
+        <is>
+          <t>Frontend cuando usuario no-admin crea porra</t>
+        </is>
+      </c>
+      <c r="C14" s="35" t="inlineStr">
+        <is>
+          <t>Supabase DB (leagues, league_members)</t>
+        </is>
+      </c>
+      <c r="D14" s="35" t="inlineStr">
+        <is>
+          <t>Permite a cualquier usuario crear una porra. Límite: 3 porras activas para no-admin. verify_jwt=false por JWT ES256 (ERR-16) — valida manualmente.</t>
+        </is>
+      </c>
+      <c r="E14" s="35" t="inlineStr">
+        <is>
+          <t>✅ En producción</t>
         </is>
       </c>
     </row>
@@ -956,6 +1069,14 @@
     <mergeCell ref="A1:E1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter>
+    <oddHeader/>
+    <oddFooter>&amp;C&amp;B Esquema Porra Mundial 2026 &amp;R Actualizado: 20 abr 2026 (commit 0d3d636)</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
 </worksheet>
 </file>
 
@@ -982,6 +1103,11 @@
           <t>PORRA MUNDIAL 2026 — Actores Apify y Crons pg_cron</t>
         </is>
       </c>
+      <c r="B1" s="33" t="n"/>
+      <c r="C1" s="33" t="n"/>
+      <c r="D1" s="33" t="n"/>
+      <c r="E1" s="33" t="n"/>
+      <c r="F1" s="34" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -1021,6 +1147,11 @@
           <t>Actores Apify</t>
         </is>
       </c>
+      <c r="B3" s="33" t="n"/>
+      <c r="C3" s="33" t="n"/>
+      <c r="D3" s="33" t="n"/>
+      <c r="E3" s="33" t="n"/>
+      <c r="F3" s="34" t="n"/>
     </row>
     <row r="4" ht="65" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
@@ -1141,6 +1272,11 @@
           <t>pg_cron — Trabajos programados</t>
         </is>
       </c>
+      <c r="B7" s="33" t="n"/>
+      <c r="C7" s="33" t="n"/>
+      <c r="D7" s="33" t="n"/>
+      <c r="E7" s="33" t="n"/>
+      <c r="F7" s="34" t="n"/>
     </row>
     <row r="8" ht="65" customHeight="1">
       <c r="A8" s="3" t="inlineStr">
@@ -1248,6 +1384,14 @@
     <mergeCell ref="A7:F7"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter>
+    <oddHeader/>
+    <oddFooter>&amp;C&amp;B Esquema Porra Mundial 2026 &amp;R Actualizado: 20 abr 2026 (commit 0d3d636)</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
 </worksheet>
 </file>
 
@@ -1257,7 +1401,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F18"/>
+  <dimension ref="A1:F19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1274,6 +1418,11 @@
           <t>PORRA MUNDIAL 2026 — APIs Externas y Tablas Supabase</t>
         </is>
       </c>
+      <c r="B1" s="33" t="n"/>
+      <c r="C1" s="33" t="n"/>
+      <c r="D1" s="33" t="n"/>
+      <c r="E1" s="33" t="n"/>
+      <c r="F1" s="34" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -1313,6 +1462,11 @@
           <t>APIs Externas</t>
         </is>
       </c>
+      <c r="B3" s="33" t="n"/>
+      <c r="C3" s="33" t="n"/>
+      <c r="D3" s="33" t="n"/>
+      <c r="E3" s="33" t="n"/>
+      <c r="F3" s="34" t="n"/>
     </row>
     <row r="4" ht="60" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
@@ -1601,6 +1755,11 @@
           <t>Tablas Supabase clave</t>
         </is>
       </c>
+      <c r="B12" s="33" t="n"/>
+      <c r="C12" s="33" t="n"/>
+      <c r="D12" s="33" t="n"/>
+      <c r="E12" s="33" t="n"/>
+      <c r="F12" s="34" t="n"/>
     </row>
     <row r="13" ht="60" customHeight="1">
       <c r="A13" s="3" t="inlineStr">
@@ -1792,6 +1951,38 @@
         </is>
       </c>
       <c r="F18" s="5" t="inlineStr">
+        <is>
+          <t>✅ Activa</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="35" t="inlineStr">
+        <is>
+          <t>league_members</t>
+        </is>
+      </c>
+      <c r="B19" s="35" t="inlineStr">
+        <is>
+          <t>Frontend (usuario autenticado)</t>
+        </is>
+      </c>
+      <c r="C19" s="35" t="inlineStr">
+        <is>
+          <t>Supabase Postgres</t>
+        </is>
+      </c>
+      <c r="D19" s="35" t="inlineStr">
+        <is>
+          <t>Membresías de usuarios en ligas. Columnas: league_id, user_id, porra_cerrada, cerrada_at. NUEVO 19abr26: groups_saved JSONB DEFAULT '{}' — mapa {A:true...}. Policy lm_update requiere porra_cerrada=false.</t>
+        </is>
+      </c>
+      <c r="E19" s="35" t="inlineStr">
+        <is>
+          <t>RLS Supabase</t>
+        </is>
+      </c>
+      <c r="F19" s="35" t="inlineStr">
         <is>
           <t>✅ Activa</t>
         </is>
@@ -1804,6 +1995,14 @@
     <mergeCell ref="A12:F12"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter>
+    <oddHeader/>
+    <oddFooter>&amp;C&amp;B Esquema Porra Mundial 2026 &amp;R Actualizado: 20 abr 2026 (commit 0d3d636)</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
 </worksheet>
 </file>
 
@@ -1828,6 +2027,9 @@
           <t>FLUJO COMPLETO — Sistema live scores + notificaciones WhatsApp (arquitectura ASYNC+WEBHOOK)</t>
         </is>
       </c>
+      <c r="B1" s="33" t="n"/>
+      <c r="C1" s="33" t="n"/>
+      <c r="D1" s="34" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -2210,6 +2412,9 @@
           <t>⚠️ ROLLBACK: Si Webshare falla → en porra-match-live cambiar ACTOR_ID = 'N8vUChlhok5JU3cnL' por 'BYLtYcOxYkruVipwr'</t>
         </is>
       </c>
+      <c r="B20" s="33" t="n"/>
+      <c r="C20" s="33" t="n"/>
+      <c r="D20" s="34" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -2217,6 +2422,9 @@
           <t>LEYENDA DE ESTADOS</t>
         </is>
       </c>
+      <c r="B22" s="33" t="n"/>
+      <c r="C22" s="33" t="n"/>
+      <c r="D22" s="34" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
@@ -2229,6 +2437,8 @@
           <t>Componente operativo y probado</t>
         </is>
       </c>
+      <c r="C23" s="33" t="n"/>
+      <c r="D23" s="34" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="17" t="inlineStr">
@@ -2241,6 +2451,8 @@
           <t>Funciona pero no activo actualmente (disponible para rollback)</t>
         </is>
       </c>
+      <c r="C24" s="33" t="n"/>
+      <c r="D24" s="34" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="11" t="inlineStr">
@@ -2253,6 +2465,8 @@
           <t>Componente descartado</t>
         </is>
       </c>
+      <c r="C25" s="33" t="n"/>
+      <c r="D25" s="34" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="8" t="inlineStr">
@@ -2265,6 +2479,8 @@
           <t>Configurado pero no activo todavía (espera fecha o condición)</t>
         </is>
       </c>
+      <c r="C26" s="33" t="n"/>
+      <c r="D26" s="34" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="7">
@@ -2277,6 +2493,14 @@
     <mergeCell ref="B24:D24"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter>
+    <oddHeader/>
+    <oddFooter>&amp;C&amp;B Esquema Porra Mundial 2026 &amp;R Actualizado: 20 abr 2026 (commit 0d3d636)</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
 </worksheet>
 </file>
 
@@ -2301,6 +2525,9 @@
           <t>PORRA MUNDIAL 2026 — IDs SofaScore + Estimación de Costes</t>
         </is>
       </c>
+      <c r="B1" s="33" t="n"/>
+      <c r="C1" s="33" t="n"/>
+      <c r="D1" s="34" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -2478,6 +2705,9 @@
           <t>Estimación de costes — Mundial 2026 completo</t>
         </is>
       </c>
+      <c r="B14" s="33" t="n"/>
+      <c r="C14" s="33" t="n"/>
+      <c r="D14" s="34" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="28" t="inlineStr">
@@ -2576,6 +2806,9 @@
           <t>Desglose actual (con Webshare)</t>
         </is>
       </c>
+      <c r="B20" s="33" t="n"/>
+      <c r="C20" s="33" t="n"/>
+      <c r="D20" s="34" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
@@ -2653,5 +2886,1367 @@
     <mergeCell ref="A14:D14"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter>
+    <oddHeader/>
+    <oddFooter>&amp;C&amp;B Esquema Porra Mundial 2026 &amp;R Actualizado: 20 abr 2026 (commit 0d3d636)</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D41"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="45" customWidth="1" min="3" max="3"/>
+    <col width="55" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="36" t="inlineStr">
+        <is>
+          <t>PORRA MUNDIAL 2026 — Frontend móvil (feat/mobile-grupos-focus merged 19abr26)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="37" t="inlineStr">
+        <is>
+          <t>MÓDULOS JS — public/js/</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Módulo</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Líneas</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Rol</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Notas</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="35" t="inlineStr">
+        <is>
+          <t>main-entry.js</t>
+        </is>
+      </c>
+      <c r="B5" s="35" t="inlineStr">
+        <is>
+          <t>~20</t>
+        </is>
+      </c>
+      <c r="C5" s="35" t="inlineStr">
+        <is>
+          <t>Entry point Vite type=module</t>
+        </is>
+      </c>
+      <c r="D5" s="35" t="inlineStr">
+        <is>
+          <t>Bootstrap clásico — dispara carga ordenada</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="35" t="inlineStr">
+        <is>
+          <t>data.js</t>
+        </is>
+      </c>
+      <c r="B6" s="35" t="inlineStr">
+        <is>
+          <t>215</t>
+        </is>
+      </c>
+      <c r="C6" s="35" t="inlineStr">
+        <is>
+          <t>Datos torneo + estado global</t>
+        </is>
+      </c>
+      <c r="D6" s="35" t="inlineStr">
+        <is>
+          <t>EQUIPOS, PARTIDOS, PHRASES_GRUPO, boostPicks, groupSaved</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="35" t="inlineStr">
+        <is>
+          <t>scoring.js</t>
+        </is>
+      </c>
+      <c r="B7" s="35" t="inlineStr">
+        <is>
+          <t>1184</t>
+        </is>
+      </c>
+      <c r="C7" s="35" t="inlineStr">
+        <is>
+          <t>Motor puntos + tarjetas + premios</t>
+        </is>
+      </c>
+      <c r="D7" s="35" t="inlineStr">
+        <is>
+          <t>renderMatchCard, updateCardUI, AWARDS_CFG</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="35" t="inlineStr">
+        <is>
+          <t>ui-groups.js</t>
+        </is>
+      </c>
+      <c r="B8" s="35" t="inlineStr">
+        <is>
+          <t>167</t>
+        </is>
+      </c>
+      <c r="C8" s="35" t="inlineStr">
+        <is>
+          <t>Grupos + vista Jornada</t>
+        </is>
+      </c>
+      <c r="D8" s="35" t="inlineStr">
+        <is>
+          <t>renderGroups, tarjetas compactas jornada</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="35" t="inlineStr">
+        <is>
+          <t>ui-groups-mobile.js</t>
+        </is>
+      </c>
+      <c r="B9" s="35" t="inlineStr">
+        <is>
+          <t>~700</t>
+        </is>
+      </c>
+      <c r="C9" s="35" t="inlineStr">
+        <is>
+          <t>Acordeón + focus layer + carrusel</t>
+        </is>
+      </c>
+      <c r="D9" s="38" t="inlineStr">
+        <is>
+          <t>NUEVO 19abr26. ensureFocusLayer, openMobileFocus, smart boost, slide 7, guardar async</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="35" t="inlineStr">
+        <is>
+          <t>ko.js</t>
+        </is>
+      </c>
+      <c r="B10" s="35" t="inlineStr">
+        <is>
+          <t>1048</t>
+        </is>
+      </c>
+      <c r="C10" s="35" t="inlineStr">
+        <is>
+          <t>Bracket KO + IA</t>
+        </is>
+      </c>
+      <c r="D10" s="35" t="inlineStr">
+        <is>
+          <t>Fase eliminatoria</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="35" t="inlineStr">
+        <is>
+          <t>ui-nav.js</t>
+        </is>
+      </c>
+      <c r="B11" s="35" t="inlineStr">
+        <is>
+          <t>653</t>
+        </is>
+      </c>
+      <c r="C11" s="35" t="inlineStr">
+        <is>
+          <t>SPA nav + modal + welcome</t>
+        </is>
+      </c>
+      <c r="D11" s="35" t="inlineStr">
+        <is>
+          <t>showPage</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="35" t="inlineStr">
+        <is>
+          <t>auth.js</t>
+        </is>
+      </c>
+      <c r="B12" s="35" t="inlineStr">
+        <is>
+          <t>~400</t>
+        </is>
+      </c>
+      <c r="C12" s="35" t="inlineStr">
+        <is>
+          <t>Auth Supabase</t>
+        </is>
+      </c>
+      <c r="D12" s="38" t="inlineStr">
+        <is>
+          <t>NUEVO 19abr26: 4ª query Promise.all a league_members.groups_saved</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="35" t="inlineStr">
+        <is>
+          <t>leagues.js</t>
+        </is>
+      </c>
+      <c r="B13" s="35" t="inlineStr">
+        <is>
+          <t>~300</t>
+        </is>
+      </c>
+      <c r="C13" s="35" t="inlineStr">
+        <is>
+          <t>Ligas</t>
+        </is>
+      </c>
+      <c r="D13" s="35" t="inlineStr">
+        <is>
+          <t>Multi-liga, código invitación</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="35" t="inlineStr">
+        <is>
+          <t>misc.js</t>
+        </is>
+      </c>
+      <c r="B14" s="35" t="inlineStr">
+        <is>
+          <t>~200</t>
+        </is>
+      </c>
+      <c r="C14" s="35" t="inlineStr">
+        <is>
+          <t>Utils UI (paralelo)</t>
+        </is>
+      </c>
+      <c r="D14" s="35" t="inlineStr">
+        <is>
+          <t>showToast, lockUI</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="35" t="inlineStr">
+        <is>
+          <t>scoreboard.js</t>
+        </is>
+      </c>
+      <c r="B15" s="35" t="inlineStr">
+        <is>
+          <t>~250</t>
+        </is>
+      </c>
+      <c r="C15" s="35" t="inlineStr">
+        <is>
+          <t>Clasificación</t>
+        </is>
+      </c>
+      <c r="D15" s="35" t="inlineStr">
+        <is>
+          <t>Ranking porras</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="35" t="inlineStr">
+        <is>
+          <t>close-porra.js</t>
+        </is>
+      </c>
+      <c r="B16" s="35" t="inlineStr">
+        <is>
+          <t>~100</t>
+        </is>
+      </c>
+      <c r="C16" s="35" t="inlineStr">
+        <is>
+          <t>Cierre pronósticos</t>
+        </is>
+      </c>
+      <c r="D16" s="35" t="inlineStr">
+        <is>
+          <t>Bloqueo al cerrar</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="35" t="inlineStr">
+        <is>
+          <t>admin.js</t>
+        </is>
+      </c>
+      <c r="B17" s="35" t="inlineStr">
+        <is>
+          <t>~500</t>
+        </is>
+      </c>
+      <c r="C17" s="35" t="inlineStr">
+        <is>
+          <t>Panel admin + dados</t>
+        </is>
+      </c>
+      <c r="D17" s="35" t="inlineStr">
+        <is>
+          <t>dice.js integrado</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="35" t="inlineStr">
+        <is>
+          <t>bracket-results.js</t>
+        </is>
+      </c>
+      <c r="B18" s="35" t="inlineStr">
+        <is>
+          <t>~300</t>
+        </is>
+      </c>
+      <c r="C18" s="35" t="inlineStr">
+        <is>
+          <t>Vista resultados KO</t>
+        </is>
+      </c>
+      <c r="D18" s="35" t="inlineStr">
+        <is>
+          <t>Mobile min-width 260px</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="35" t="inlineStr">
+        <is>
+          <t>live-sync.js</t>
+        </is>
+      </c>
+      <c r="B19" s="35" t="inlineStr">
+        <is>
+          <t>~150</t>
+        </is>
+      </c>
+      <c r="C19" s="35" t="inlineStr">
+        <is>
+          <t>Sync live scores</t>
+        </is>
+      </c>
+      <c r="D19" s="35" t="inlineStr">
+        <is>
+          <t>Realtime Supabase</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="35" t="inlineStr">
+        <is>
+          <t>ui-directo.js</t>
+        </is>
+      </c>
+      <c r="B20" s="35" t="inlineStr">
+        <is>
+          <t>~200</t>
+        </is>
+      </c>
+      <c r="C20" s="35" t="inlineStr">
+        <is>
+          <t>Vista Directo</t>
+        </is>
+      </c>
+      <c r="D20" s="35" t="inlineStr">
+        <is>
+          <t>Panel live partidos simultáneos</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="37" t="inlineStr">
+        <is>
+          <t>CSS público — public/css/ (7 ficheros linkeados desde index.html tras refactor 9e93fe8)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>Fichero</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Tamaño aprox</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>Rol</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>Notas</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="35" t="inlineStr">
+        <is>
+          <t>base.css</t>
+        </is>
+      </c>
+      <c r="B24" s="35" t="inlineStr">
+        <is>
+          <t>67 KB</t>
+        </is>
+      </c>
+      <c r="C24" s="35" t="inlineStr">
+        <is>
+          <t>Base + acordeón móvil + focus layer</t>
+        </is>
+      </c>
+      <c r="D24" s="35" t="inlineStr">
+        <is>
+          <t>mobile-collapsed, mobile-focus-layer (fuera @media), smart boost</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="35" t="inlineStr">
+        <is>
+          <t>welcome.css</t>
+        </is>
+      </c>
+      <c r="B25" s="35" t="inlineStr">
+        <is>
+          <t>22 KB</t>
+        </is>
+      </c>
+      <c r="C25" s="35" t="inlineStr">
+        <is>
+          <t>Pantalla splash/welcome</t>
+        </is>
+      </c>
+      <c r="D25" s="35" t="inlineStr">
+        <is>
+          <t>Hero + scroll-cue</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="35" t="inlineStr">
+        <is>
+          <t>ko.css</t>
+        </is>
+      </c>
+      <c r="B26" s="35" t="inlineStr">
+        <is>
+          <t>64 KB</t>
+        </is>
+      </c>
+      <c r="C26" s="35" t="inlineStr">
+        <is>
+          <t>Fase eliminatoria + awards</t>
+        </is>
+      </c>
+      <c r="D26" s="35" t="inlineStr">
+        <is>
+          <t>Bracket KO, cards premios individuales</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="35" t="inlineStr">
+        <is>
+          <t>admin.css</t>
+        </is>
+      </c>
+      <c r="B27" s="35" t="inlineStr">
+        <is>
+          <t>57 KB</t>
+        </is>
+      </c>
+      <c r="C27" s="35" t="inlineStr">
+        <is>
+          <t>Panel administrador</t>
+        </is>
+      </c>
+      <c r="D27" s="35" t="inlineStr">
+        <is>
+          <t>Dados, simulador, simulacros</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="35" t="inlineStr">
+        <is>
+          <t>bracket-results.css</t>
+        </is>
+      </c>
+      <c r="B28" s="35" t="inlineStr">
+        <is>
+          <t>~15 KB</t>
+        </is>
+      </c>
+      <c r="C28" s="35" t="inlineStr">
+        <is>
+          <t>Vista resultados KO</t>
+        </is>
+      </c>
+      <c r="D28" s="35" t="inlineStr">
+        <is>
+          <t>Mobile: min-width 260px columna activa</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="35" t="inlineStr">
+        <is>
+          <t>boost.css</t>
+        </is>
+      </c>
+      <c r="B29" s="35" t="inlineStr">
+        <is>
+          <t>~10 KB</t>
+        </is>
+      </c>
+      <c r="C29" s="35" t="inlineStr">
+        <is>
+          <t>Boost x2 fuego canvas</t>
+        </is>
+      </c>
+      <c r="D29" s="35" t="inlineStr">
+        <is>
+          <t>Ticker boosts, efecto Canvas</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="35" t="inlineStr">
+        <is>
+          <t>directo.css</t>
+        </is>
+      </c>
+      <c r="B30" s="35" t="inlineStr">
+        <is>
+          <t>~12 KB</t>
+        </is>
+      </c>
+      <c r="C30" s="35" t="inlineStr">
+        <is>
+          <t>Vista Directo live</t>
+        </is>
+      </c>
+      <c r="D30" s="35" t="inlineStr">
+        <is>
+          <t>Panel en vivo, pills CEST</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="37" t="inlineStr">
+        <is>
+          <t>Rediseño móvil grupos — componentes (PR#9 → refactor CSS 9e93fe8)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>Componente</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>Activación</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>Descripción</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>Persistencia</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="35" t="inlineStr">
+        <is>
+          <t>Acordeón colapsado</t>
+        </is>
+      </c>
+      <c r="B34" s="35" t="inlineStr">
+        <is>
+          <t>Viewport ≤640px</t>
+        </is>
+      </c>
+      <c r="C34" s="35" t="inlineStr">
+        <is>
+          <t>Grupos plegados con header + barra progreso</t>
+        </is>
+      </c>
+      <c r="D34" s="35" t="inlineStr">
+        <is>
+          <t>Estado memoria</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="35" t="inlineStr">
+        <is>
+          <t>Focus layer pantalla completa</t>
+        </is>
+      </c>
+      <c r="B35" s="35" t="inlineStr">
+        <is>
+          <t>Tap en header grupo</t>
+        </is>
+      </c>
+      <c r="C35" s="35" t="inlineStr">
+        <is>
+          <t>position:fixed inset:0 z-index:100. 7 slides</t>
+        </is>
+      </c>
+      <c r="D35" s="35" t="inlineStr">
+        <is>
+          <t>__mobileFocusState</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="35" t="inlineStr">
+        <is>
+          <t>Carrusel tarjetas</t>
+        </is>
+      </c>
+      <c r="B36" s="35" t="inlineStr">
+        <is>
+          <t>Dentro focus layer</t>
+        </is>
+      </c>
+      <c r="C36" s="35" t="inlineStr">
+        <is>
+          <t>6 tarjetas + slide 7 summary. Swipe threshold 50px. Dots + flechas</t>
+        </is>
+      </c>
+      <c r="D36" s="35" t="inlineStr">
+        <is>
+          <t>__mobileFocusState.slide</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="35" t="inlineStr">
+        <is>
+          <t>Smart boost multi-jornada</t>
+        </is>
+      </c>
+      <c r="B37" s="35" t="inlineStr">
+        <is>
+          <t>Botón boost</t>
+        </is>
+      </c>
+      <c r="C37" s="35" t="inlineStr">
+        <is>
+          <t>Detecta conflictos inter-grupo mismo match_date. confirm() si conflicto</t>
+        </is>
+      </c>
+      <c r="D37" s="35" t="inlineStr">
+        <is>
+          <t>boost_picks tabla</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="35" t="inlineStr">
+        <is>
+          <t>Slide 7 summary</t>
+        </is>
+      </c>
+      <c r="B38" s="35" t="inlineStr">
+        <is>
+          <t>Slide final</t>
+        </is>
+      </c>
+      <c r="C38" s="35" t="inlineStr">
+        <is>
+          <t>Mueve #gtable-L al slide. Fallback si falta tabla</t>
+        </is>
+      </c>
+      <c r="D38" s="35" t="inlineStr">
+        <is>
+          <t>Tabla del grupo</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="35" t="inlineStr">
+        <is>
+          <t>Guardar/deshacer</t>
+        </is>
+      </c>
+      <c r="B39" s="35" t="inlineStr">
+        <is>
+          <t>💾 Guardar grupo</t>
+        </is>
+      </c>
+      <c r="C39" s="35" t="inlineStr">
+        <is>
+          <t>4 estados: guardar/guardado/deshacer/bloqueado. canSaveGroup verifica 6 partidos</t>
+        </is>
+      </c>
+      <c r="D39" s="35" t="inlineStr">
+        <is>
+          <t>league_members.groups_saved JSONB</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="35" t="inlineStr">
+        <is>
+          <t>Barra progreso grupo</t>
+        </is>
+      </c>
+      <c r="B40" s="35" t="inlineStr">
+        <is>
+          <t>Header colapsado</t>
+        </is>
+      </c>
+      <c r="C40" s="35" t="inlineStr">
+        <is>
+          <t>Cuenta partidos con pred. completa</t>
+        </is>
+      </c>
+      <c r="D40" s="35" t="inlineStr">
+        <is>
+          <t>Estado memoria</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="35" t="inlineStr">
+        <is>
+          <t>Frase motivacional</t>
+        </is>
+      </c>
+      <c r="B41" s="35" t="inlineStr">
+        <is>
+          <t>Header focus</t>
+        </is>
+      </c>
+      <c r="C41" s="35" t="inlineStr">
+        <is>
+          <t>PHRASES_GRUPO[letra][percent] varía según completitud</t>
+        </is>
+      </c>
+      <c r="D41" s="35" t="inlineStr">
+        <is>
+          <t>data.js</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="A22:D22"/>
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A32:D32"/>
+    <mergeCell ref="A3:D3"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter>
+    <oddHeader/>
+    <oddFooter>&amp;C&amp;B Esquema Porra Mundial 2026 &amp;R Actualizado: 20 abr 2026 (commit 0d3d636)</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D25"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="45" customWidth="1" min="2" max="2"/>
+    <col width="45" customWidth="1" min="3" max="3"/>
+    <col width="55" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="36" t="inlineStr">
+        <is>
+          <t>PORRA MUNDIAL 2026 — Inventario de errores conocidos</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Síntoma</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Causa raíz</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Fix</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="35" t="inlineStr">
+        <is>
+          <t>ERR-01</t>
+        </is>
+      </c>
+      <c r="B4" s="35" t="inlineStr">
+        <is>
+          <t>DOMContentLoaded no dispara en classic scripts async</t>
+        </is>
+      </c>
+      <c r="C4" s="35" t="inlineStr">
+        <is>
+          <t>Script ya cargado cuando registras listener</t>
+        </is>
+      </c>
+      <c r="D4" s="35" t="inlineStr">
+        <is>
+          <t>if (document.readyState===loading) addEventListener else run()</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="35" t="inlineStr">
+        <is>
+          <t>ERR-02</t>
+        </is>
+      </c>
+      <c r="B5" s="35" t="inlineStr">
+        <is>
+          <t>const globals no accesibles entre módulos</t>
+        </is>
+      </c>
+      <c r="C5" s="35" t="inlineStr">
+        <is>
+          <t>const no se expone en window automáticamente</t>
+        </is>
+      </c>
+      <c r="D5" s="35" t="inlineStr">
+        <is>
+          <t>window.X = X explícito</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="35" t="inlineStr">
+        <is>
+          <t>ERR-03</t>
+        </is>
+      </c>
+      <c r="B6" s="35" t="inlineStr">
+        <is>
+          <t>Vite no copia assets de /css en build</t>
+        </is>
+      </c>
+      <c r="C6" s="35" t="inlineStr">
+        <is>
+          <t>Vite solo copia public/</t>
+        </is>
+      </c>
+      <c r="D6" s="35" t="inlineStr">
+        <is>
+          <t>Mover css/ → public/css/</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="35" t="inlineStr">
+        <is>
+          <t>ERR-04</t>
+        </is>
+      </c>
+      <c r="B7" s="35" t="inlineStr">
+        <is>
+          <t>Whitespace en secrets Vault rompe HTTP</t>
+        </is>
+      </c>
+      <c r="C7" s="35" t="inlineStr">
+        <is>
+          <t>Secrets con newline al final</t>
+        </is>
+      </c>
+      <c r="D7" s="35" t="inlineStr">
+        <is>
+          <t>trim() antes de usar</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="35" t="inlineStr">
+        <is>
+          <t>ERR-05</t>
+        </is>
+      </c>
+      <c r="B8" s="35" t="inlineStr">
+        <is>
+          <t>pg_net timeout &gt;30s</t>
+        </is>
+      </c>
+      <c r="C8" s="35" t="inlineStr">
+        <is>
+          <t>Timeout fijo ~30s</t>
+        </is>
+      </c>
+      <c r="D8" s="35" t="inlineStr">
+        <is>
+          <t>Async + webhook pattern</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="35" t="inlineStr">
+        <is>
+          <t>ERR-06</t>
+        </is>
+      </c>
+      <c r="B9" s="35" t="inlineStr">
+        <is>
+          <t>vercel.json rompe MIME ES modules</t>
+        </is>
+      </c>
+      <c r="C9" s="35" t="inlineStr">
+        <is>
+          <t>Wildcard source sobrescribe Content-Type</t>
+        </is>
+      </c>
+      <c r="D9" s="35" t="inlineStr">
+        <is>
+          <t>NO crear vercel.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="35" t="inlineStr">
+        <is>
+          <t>ERR-07</t>
+        </is>
+      </c>
+      <c r="B10" s="35" t="inlineStr">
+        <is>
+          <t>GitHub raw bloqueado proxy Claude.ai</t>
+        </is>
+      </c>
+      <c r="C10" s="35" t="inlineStr">
+        <is>
+          <t>Dominio no whitelisted</t>
+        </is>
+      </c>
+      <c r="D10" s="35" t="inlineStr">
+        <is>
+          <t>net.http_post + GITHUB_TOKEN desde Supabase MCP</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="35" t="inlineStr">
+        <is>
+          <t>ERR-08</t>
+        </is>
+      </c>
+      <c r="B11" s="35" t="inlineStr">
+        <is>
+          <t>SofaScore API 403 (Cloudflare)</t>
+        </is>
+      </c>
+      <c r="C11" s="35" t="inlineStr">
+        <is>
+          <t>Bot Management detecta peticiones no-browser</t>
+        </is>
+      </c>
+      <c r="D11" s="35" t="inlineStr">
+        <is>
+          <t>Playwright proxy residencial + page.evaluate(fetch)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="35" t="inlineStr">
+        <is>
+          <t>ERR-09</t>
+        </is>
+      </c>
+      <c r="B12" s="35" t="inlineStr">
+        <is>
+          <t>checkIsAdmin async no detecta admin render inicial</t>
+        </is>
+      </c>
+      <c r="C12" s="35" t="inlineStr">
+        <is>
+          <t>Race condition render vs query profiles</t>
+        </is>
+      </c>
+      <c r="D12" s="35" t="inlineStr">
+        <is>
+          <t>Retries + re-render al completar</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="35" t="inlineStr">
+        <is>
+          <t>ERR-10</t>
+        </is>
+      </c>
+      <c r="B13" s="35" t="inlineStr">
+        <is>
+          <t>Webhook Apify no llega</t>
+        </is>
+      </c>
+      <c r="C13" s="35" t="inlineStr">
+        <is>
+          <t>Filtro eventTypes incorrecto</t>
+        </is>
+      </c>
+      <c r="D13" s="35" t="inlineStr">
+        <is>
+          <t>ACTOR.RUN.SUCCEEDED + FAILED</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="35" t="inlineStr">
+        <is>
+          <t>ERR-11</t>
+        </is>
+      </c>
+      <c r="B14" s="35" t="inlineStr">
+        <is>
+          <t>Twilio 21211 invalid To</t>
+        </is>
+      </c>
+      <c r="C14" s="35" t="inlineStr">
+        <is>
+          <t>Falta prefijo whatsapp:</t>
+        </is>
+      </c>
+      <c r="D14" s="35" t="inlineStr">
+        <is>
+          <t>whatsapp:+34XXX</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="35" t="inlineStr">
+        <is>
+          <t>ERR-12</t>
+        </is>
+      </c>
+      <c r="B15" s="35" t="inlineStr">
+        <is>
+          <t>porra-whatsapp-send pg_net 400</t>
+        </is>
+      </c>
+      <c r="C15" s="35" t="inlineStr">
+        <is>
+          <t>pg_net no soporta form-urlencoded</t>
+        </is>
+      </c>
+      <c r="D15" s="35" t="inlineStr">
+        <is>
+          <t>fetch() Content-Type x-www-form-urlencoded</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="35" t="inlineStr">
+        <is>
+          <t>ERR-13</t>
+        </is>
+      </c>
+      <c r="B16" s="35" t="inlineStr">
+        <is>
+          <t>porra-fix-encoding 404 intermitente</t>
+        </is>
+      </c>
+      <c r="C16" s="35" t="inlineStr">
+        <is>
+          <t>Reuso conexión EF antigua</t>
+        </is>
+      </c>
+      <c r="D16" s="35" t="inlineStr">
+        <is>
+          <t>Retry 5-10s</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="35" t="inlineStr">
+        <is>
+          <t>ERR-14</t>
+        </is>
+      </c>
+      <c r="B17" s="35" t="inlineStr">
+        <is>
+          <t>Simulacro admin no aparece al cargar</t>
+        </is>
+      </c>
+      <c r="C17" s="35" t="inlineStr">
+        <is>
+          <t>checkIsAdmin async no completa antes render</t>
+        </is>
+      </c>
+      <c r="D17" s="35" t="inlineStr">
+        <is>
+          <t>Retry 3x + re-render</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="35" t="inlineStr">
+        <is>
+          <t>ERR-15</t>
+        </is>
+      </c>
+      <c r="B18" s="35" t="inlineStr">
+        <is>
+          <t>QA sobrescribir encrypted_password invalida sesiones</t>
+        </is>
+      </c>
+      <c r="C18" s="35" t="inlineStr">
+        <is>
+          <t>Manipular auth.users rompe Supabase Auth</t>
+        </is>
+      </c>
+      <c r="D18" s="35" t="inlineStr">
+        <is>
+          <t>generateLink para reset</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="35" t="inlineStr">
+        <is>
+          <t>ERR-16</t>
+        </is>
+      </c>
+      <c r="B19" s="35" t="inlineStr">
+        <is>
+          <t>EF verify_jwt=true falla con JWT ES256</t>
+        </is>
+      </c>
+      <c r="C19" s="35" t="inlineStr">
+        <is>
+          <t>Supabase no valida ES256 automáticamente</t>
+        </is>
+      </c>
+      <c r="D19" s="35" t="inlineStr">
+        <is>
+          <t>verify_jwt=false + jose manual</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="35" t="inlineStr">
+        <is>
+          <t>ERR-17</t>
+        </is>
+      </c>
+      <c r="B20" s="35" t="inlineStr">
+        <is>
+          <t>net.http_put no existe en pg_net</t>
+        </is>
+      </c>
+      <c r="C20" s="35" t="inlineStr">
+        <is>
+          <t>pg_net solo GET/POST/DELETE</t>
+        </is>
+      </c>
+      <c r="D20" s="35" t="inlineStr">
+        <is>
+          <t>Chrome MCP para merge PR</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="39" t="inlineStr">
+        <is>
+          <t>ERR-18</t>
+        </is>
+      </c>
+      <c r="B21" s="39" t="inlineStr">
+        <is>
+          <t>css/ no servido prod tras merge</t>
+        </is>
+      </c>
+      <c r="C21" s="39" t="inlineStr">
+        <is>
+          <t>Vite no copia /css/ del root</t>
+        </is>
+      </c>
+      <c r="D21" s="39" t="inlineStr">
+        <is>
+          <t>Mover a public/css/. Parcial — real era ERR-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="39" t="inlineStr">
+        <is>
+          <t>ERR-19</t>
+        </is>
+      </c>
+      <c r="B22" s="39" t="inlineStr">
+        <is>
+          <t>openMobileFocus sin try/catch deja body inconsistente</t>
+        </is>
+      </c>
+      <c r="C22" s="39" t="inlineStr">
+        <is>
+          <t>body.overflow=hidden antes de confirmar éxito</t>
+        </is>
+      </c>
+      <c r="D22" s="39" t="inlineStr">
+        <is>
+          <t>try/catch + overflow al final (después eliminado)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="39" t="inlineStr">
+        <is>
+          <t>ERR-20</t>
+        </is>
+      </c>
+      <c r="B23" s="39" t="inlineStr">
+        <is>
+          <t>body.overflow=hidden bloquea scroll iPhone Safari</t>
+        </is>
+      </c>
+      <c r="C23" s="39" t="inlineStr">
+        <is>
+          <t>WebKit iOS quirk persistente</t>
+        </is>
+      </c>
+      <c r="D23" s="39" t="inlineStr">
+        <is>
+          <t>Eliminar uso de body.overflow=hidden. position:fixed basta</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="39" t="inlineStr">
+        <is>
+          <t>ERR-21</t>
+        </is>
+      </c>
+      <c r="B24" s="39" t="inlineStr">
+        <is>
+          <t>.mobile-focus-layer inline en viewport &gt;640px</t>
+        </is>
+      </c>
+      <c r="C24" s="39" t="inlineStr">
+        <is>
+          <t>Reglas CSS dentro @media</t>
+        </is>
+      </c>
+      <c r="D24" s="39" t="inlineStr">
+        <is>
+          <t>Sacar base del @media + visibility:hidden/visible</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="39" t="inlineStr">
+        <is>
+          <t>ERR-22</t>
+        </is>
+      </c>
+      <c r="B25" s="39" t="inlineStr">
+        <is>
+          <t>Reglas CSS nuevas NO aplican prod (root cause real)</t>
+        </is>
+      </c>
+      <c r="C25" s="39" t="inlineStr">
+        <is>
+          <t>index.html tenía &lt;style&gt; inline con "Archivo destino:X.css" nunca migrados. &lt;link&gt; no existían</t>
+        </is>
+      </c>
+      <c r="D25" s="39" t="inlineStr">
+        <is>
+          <t>Refactor commit 9e93fe8: extraer &lt;style&gt; → public/css/ + 4 &lt;link&gt; en &lt;head&gt;. getComputedStyle() test definitivo</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:D1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter>
+    <oddHeader/>
+    <oddFooter>&amp;C&amp;B Esquema Porra Mundial 2026 &amp;R Actualizado: 20 abr 2026 (commit 0d3d636)</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs(checkpoint): fin sesión 20abr noche — persistencia última página
Saga v2.1→v2.11 estable tras 11 iteraciones. HEAD funcional 8bc7f30.

CLAUDE.md: cabecera + cierre bug parpadeo botón envío + sección
'Persistencia última página al F5' con diagrama de arranque y limitaciones.

CONTEXTO_PORRA_2026.md: cabecera + entrada en historial sesiones.

migration-log.md: entrada única consolidando estado vigente, capas
defensivas, ficheros tocados, commits revertidos (sin detallar reverts).

errores_conocidos_porra.md: ERR-23 nuevo (ERR-22 ya estaba ocupado por
migración CSS inline de la sesión 19abr). Diagnóstico definitivo +
las 5 capas de causas + solución belt & suspenders + lecciones.

ESQUEMA_SISTEMA_PORRA2026.xlsx: hoja 'Errores ERR-01..ERR-22' renombrada
a ERR-01..ERR-23. Fila ERR-23 añadida. Sección nueva en Frontend Mobile
con las 6 capas de la persistencia. Footer actualizado a HEAD 8bc7f30.
</commit_message>
<xml_diff>
--- a/ESQUEMA_SISTEMA_PORRA2026.xlsx
+++ b/ESQUEMA_SISTEMA_PORRA2026.xlsx
@@ -13,7 +13,7 @@
     <sheet name="Flujo + Leyenda" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="IDs SofaScore + Costes" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Frontend Mobile" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Errores ERR-01..ERR-22" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Errores ERR-01..ERR-23" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1071,7 +1071,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;C&amp;B Esquema Porra Mundial 2026 &amp;R Actualizado: 20 abr 2026 (commit 0d3d636)</oddFooter>
+    <oddFooter>&amp;C&amp;B Esquema Porra Mundial 2026 &amp;R Actualizado: 20 abr 2026 noche (HEAD 8bc7f30)&amp;R Actualizado: 20 abr 2026 (commit 0d3d636)</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -1386,7 +1386,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;C&amp;B Esquema Porra Mundial 2026 &amp;R Actualizado: 20 abr 2026 (commit 0d3d636)</oddFooter>
+    <oddFooter>&amp;C&amp;B Esquema Porra Mundial 2026 &amp;R Actualizado: 20 abr 2026 noche (HEAD 8bc7f30)&amp;R Actualizado: 20 abr 2026 (commit 0d3d636)</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -1997,7 +1997,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;C&amp;B Esquema Porra Mundial 2026 &amp;R Actualizado: 20 abr 2026 (commit 0d3d636)</oddFooter>
+    <oddFooter>&amp;C&amp;B Esquema Porra Mundial 2026 &amp;R Actualizado: 20 abr 2026 noche (HEAD 8bc7f30)&amp;R Actualizado: 20 abr 2026 (commit 0d3d636)</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -2495,7 +2495,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;C&amp;B Esquema Porra Mundial 2026 &amp;R Actualizado: 20 abr 2026 (commit 0d3d636)</oddFooter>
+    <oddFooter>&amp;C&amp;B Esquema Porra Mundial 2026 &amp;R Actualizado: 20 abr 2026 noche (HEAD 8bc7f30)&amp;R Actualizado: 20 abr 2026 (commit 0d3d636)</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -2888,7 +2888,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;C&amp;B Esquema Porra Mundial 2026 &amp;R Actualizado: 20 abr 2026 (commit 0d3d636)</oddFooter>
+    <oddFooter>&amp;C&amp;B Esquema Porra Mundial 2026 &amp;R Actualizado: 20 abr 2026 noche (HEAD 8bc7f30)&amp;R Actualizado: 20 abr 2026 (commit 0d3d636)</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -2903,7 +2903,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D41"/>
+  <dimension ref="A1:D50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -3688,17 +3688,179 @@
         </is>
       </c>
     </row>
+    <row r="43">
+      <c r="A43" s="37" t="inlineStr">
+        <is>
+          <t>Persistencia última página al F5 (NUEVO 20abr26 noche, HEAD 8bc7f30)</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>Capa</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>Fichero</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>Mecanismo</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>Versión / commit</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="35" t="inlineStr">
+        <is>
+          <t>Capa 0 (HTML head)</t>
+        </is>
+      </c>
+      <c r="B45" s="35" t="inlineStr">
+        <is>
+          <t>index.html script inline</t>
+        </is>
+      </c>
+      <c r="C45" s="35" t="inlineStr">
+        <is>
+          <t>Lee localStorage.porra_lastPage → setea window._pendingPageRestore + inyecta &lt;style id=restore-lock-css&gt;#page-welcome{display:none !important}&lt;/style&gt; + skipea splash de 4s</t>
+        </is>
+      </c>
+      <c r="D45" s="35" t="inlineStr">
+        <is>
+          <t>v2.6 e28f447 + v2.8 5ef545f + v2.9 7689bcc</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="35" t="inlineStr">
+        <is>
+          <t>Capa 1 (main-entry safety-net)</t>
+        </is>
+      </c>
+      <c r="B46" s="35" t="inlineStr">
+        <is>
+          <t>js/main-entry.js L74-78</t>
+        </is>
+      </c>
+      <c r="C46" s="35" t="inlineStr">
+        <is>
+          <t>if (!window._pendingPageRestore) showPage(welcome) — impide flash desde el chain</t>
+        </is>
+      </c>
+      <c r="D46" s="35" t="inlineStr">
+        <is>
+          <t>v2.11 d4a0047</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="35" t="inlineStr">
+        <is>
+          <t>Capa 2 (showPage lock guard)</t>
+        </is>
+      </c>
+      <c r="B47" s="35" t="inlineStr">
+        <is>
+          <t>public/js/ui-nav.js showPage()</t>
+        </is>
+      </c>
+      <c r="C47" s="35" t="inlineStr">
+        <is>
+          <t>if (lock &amp;&amp; page=welcome) return; if (lock &amp;&amp; page!=welcome) lock.remove() — lock self-healing</t>
+        </is>
+      </c>
+      <c r="D47" s="35" t="inlineStr">
+        <is>
+          <t>v2.10 4214bfe</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="35" t="inlineStr">
+        <is>
+          <t>Plus auth restore</t>
+        </is>
+      </c>
+      <c r="B48" s="35" t="inlineStr">
+        <is>
+          <t>public/js/auth.js L325-339</t>
+        </is>
+      </c>
+      <c r="C48" s="35" t="inlineStr">
+        <is>
+          <t>onAuthStateChange consume _pendingPageRestore solo en INITIAL_SESSION (no SIGNED_IN). Revalidación admin explícita. setTimeout(100) único</t>
+        </is>
+      </c>
+      <c r="D48" s="35" t="inlineStr">
+        <is>
+          <t>v2.1 aade8d0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="35" t="inlineStr">
+        <is>
+          <t>Plus auth runAuthInit guard</t>
+        </is>
+      </c>
+      <c r="B49" s="35" t="inlineStr">
+        <is>
+          <t>public/js/auth.js L349</t>
+        </is>
+      </c>
+      <c r="C49" s="35" t="inlineStr">
+        <is>
+          <t>if (!window._pendingPageRestore) showPage(welcome) en arranque + fallback else por sesión caducada</t>
+        </is>
+      </c>
+      <c r="D49" s="35" t="inlineStr">
+        <is>
+          <t>v2.7 951922a</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="35" t="inlineStr">
+        <is>
+          <t>Plus HTML attr</t>
+        </is>
+      </c>
+      <c r="B50" s="35" t="inlineStr">
+        <is>
+          <t>index.html L251</t>
+        </is>
+      </c>
+      <c r="C50" s="35" t="inlineStr">
+        <is>
+          <t>&lt;div id=page-welcome style=display:none&gt; consistente con otras 4 páginas</t>
+        </is>
+      </c>
+      <c r="D50" s="35" t="inlineStr">
+        <is>
+          <t>v2.4 caaf0a0</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="5">
+    <mergeCell ref="A1:D1"/>
     <mergeCell ref="A22:D22"/>
-    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A3:D3"/>
+    <mergeCell ref="A43:D43"/>
     <mergeCell ref="A32:D32"/>
-    <mergeCell ref="A3:D3"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;C&amp;B Esquema Porra Mundial 2026 &amp;R Actualizado: 20 abr 2026 (commit 0d3d636)</oddFooter>
+    <oddFooter>&amp;C&amp;B Esquema Porra Mundial 2026 &amp;R Actualizado: 20 abr 2026 noche (HEAD 8bc7f30)&amp;R Actualizado: 20 abr 2026 (commit 0d3d636)</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -3713,7 +3875,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D25"/>
+  <dimension ref="A1:D26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4235,6 +4397,28 @@
         </is>
       </c>
     </row>
+    <row r="26">
+      <c r="A26" s="39" t="inlineStr">
+        <is>
+          <t>ERR-23</t>
+        </is>
+      </c>
+      <c r="B26" s="39" t="inlineStr">
+        <is>
+          <t>Flash welcome al F5 con sesión válida + restore (~503ms visible cazado con MutationObserver)</t>
+        </is>
+      </c>
+      <c r="C26" s="39" t="inlineStr">
+        <is>
+          <t>5 capas de causas: page-welcome sin display:none inline + splash 4s hardcoded + module bundle deferred vs scripts inline + main-entry safety-net sin guard + CSS lock retirado por showPage(welcome) rogue</t>
+        </is>
+      </c>
+      <c r="D26" s="39" t="inlineStr">
+        <is>
+          <t>Saga v2.1→v2.11 (HEAD 8bc7f30). 3 capas defensivas: HTML head script inline (CSS lock + flag + skip splash), main-entry guard, ui-nav showPage lock-aware. Plus: auth.js INITIAL_SESSION-only restore.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:D1"/>
@@ -4242,7 +4426,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;C&amp;B Esquema Porra Mundial 2026 &amp;R Actualizado: 20 abr 2026 (commit 0d3d636)</oddFooter>
+    <oddFooter>&amp;C&amp;B Esquema Porra Mundial 2026 &amp;R Actualizado: 20 abr 2026 noche (HEAD 8bc7f30)&amp;R Actualizado: 20 abr 2026 (commit 0d3d636)</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>

</xml_diff>

<commit_message>
docs(ia-predictor): consolidación Fases A-D.2 + plan Fase E/F
</commit_message>
<xml_diff>
--- a/ESQUEMA_SISTEMA_PORRA2026.xlsx
+++ b/ESQUEMA_SISTEMA_PORRA2026.xlsx
@@ -13,7 +13,8 @@
     <sheet name="Flujo + Leyenda" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="IDs SofaScore + Costes" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Frontend Mobile" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Errores ERR-01..ERR-23" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Errores ERR-01..ERR-26" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="IA Predictor" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -23,7 +24,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -74,6 +75,11 @@
       <name val="Arial"/>
       <b val="1"/>
       <sz val="12"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <sz val="10"/>
     </font>
   </fonts>
   <fills count="14">
@@ -214,7 +220,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -325,6 +331,10 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -692,7 +702,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1064,6 +1074,33 @@
         </is>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" s="38" t="inlineStr">
+        <is>
+          <t>porra-ia-compute v6</t>
+        </is>
+      </c>
+      <c r="B15" s="38" t="inlineStr">
+        <is>
+          <t>Claude.ai via SQL (scrape_*) / pg_cron futuro (compute diario)</t>
+        </is>
+      </c>
+      <c r="C15" s="38" t="inlineStr">
+        <is>
+          <t>Wikipedia MediaWiki API + 11v11.com HTML + Supabase DB (ia_* tablas)</t>
+        </is>
+      </c>
+      <c r="D15" s="38" t="inlineStr">
+        <is>
+          <t>IA Predictor (Fases A-C implementadas). Router: status / scrape_elo (Wikipedia Module:SportsRankings → ia_elo_fifa) / scrape_h2h (11v11.com/stats → ia_h2h) / scrape_last5 (11v11.com/matches → ia_last5_results) / compute (Fase E pendiente). verify_jwt=false.</t>
+        </is>
+      </c>
+      <c r="E15" s="38" t="inlineStr">
+        <is>
+          <t>✅ En producción (Fases A-C). Fase E/F pendientes.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:E1"/>
@@ -1071,7 +1108,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;C&amp;B Esquema Porra Mundial 2026 &amp;R Actualizado: 20 abr 2026 noche (HEAD 8bc7f30)&amp;R Actualizado: 20 abr 2026 (commit 0d3d636)</oddFooter>
+    <oddFooter>&amp;C&amp;B Esquema Porra Mundial 2026 &amp;R Actualizado: 21 abr 2026 (IA Predictor A-C)&amp;R Actualizado: 20 abr 2026 noche (HEAD 8bc7f30)&amp;R Actualizado: 20 abr 2026 (commit 0d3d636)</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -1386,7 +1423,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;C&amp;B Esquema Porra Mundial 2026 &amp;R Actualizado: 20 abr 2026 noche (HEAD 8bc7f30)&amp;R Actualizado: 20 abr 2026 (commit 0d3d636)</oddFooter>
+    <oddFooter>&amp;C&amp;B Esquema Porra Mundial 2026 &amp;R Actualizado: 21 abr 2026 (IA Predictor A-C)&amp;R Actualizado: 20 abr 2026 noche (HEAD 8bc7f30)&amp;R Actualizado: 20 abr 2026 (commit 0d3d636)</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -1997,7 +2034,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;C&amp;B Esquema Porra Mundial 2026 &amp;R Actualizado: 20 abr 2026 noche (HEAD 8bc7f30)&amp;R Actualizado: 20 abr 2026 (commit 0d3d636)</oddFooter>
+    <oddFooter>&amp;C&amp;B Esquema Porra Mundial 2026 &amp;R Actualizado: 21 abr 2026 (IA Predictor A-C)&amp;R Actualizado: 20 abr 2026 noche (HEAD 8bc7f30)&amp;R Actualizado: 20 abr 2026 (commit 0d3d636)</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -2495,7 +2532,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;C&amp;B Esquema Porra Mundial 2026 &amp;R Actualizado: 20 abr 2026 noche (HEAD 8bc7f30)&amp;R Actualizado: 20 abr 2026 (commit 0d3d636)</oddFooter>
+    <oddFooter>&amp;C&amp;B Esquema Porra Mundial 2026 &amp;R Actualizado: 21 abr 2026 (IA Predictor A-C)&amp;R Actualizado: 20 abr 2026 noche (HEAD 8bc7f30)&amp;R Actualizado: 20 abr 2026 (commit 0d3d636)</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -2888,7 +2925,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;C&amp;B Esquema Porra Mundial 2026 &amp;R Actualizado: 20 abr 2026 noche (HEAD 8bc7f30)&amp;R Actualizado: 20 abr 2026 (commit 0d3d636)</oddFooter>
+    <oddFooter>&amp;C&amp;B Esquema Porra Mundial 2026 &amp;R Actualizado: 21 abr 2026 (IA Predictor A-C)&amp;R Actualizado: 20 abr 2026 noche (HEAD 8bc7f30)&amp;R Actualizado: 20 abr 2026 (commit 0d3d636)</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -3860,7 +3897,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;C&amp;B Esquema Porra Mundial 2026 &amp;R Actualizado: 20 abr 2026 noche (HEAD 8bc7f30)&amp;R Actualizado: 20 abr 2026 (commit 0d3d636)</oddFooter>
+    <oddFooter>&amp;C&amp;B Esquema Porra Mundial 2026 &amp;R Actualizado: 21 abr 2026 (IA Predictor A-C)&amp;R Actualizado: 20 abr 2026 noche (HEAD 8bc7f30)&amp;R Actualizado: 20 abr 2026 (commit 0d3d636)</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -3875,7 +3912,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D26"/>
+  <dimension ref="A1:D29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -3891,6 +3928,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -4416,6 +4454,72 @@
       <c r="D26" s="39" t="inlineStr">
         <is>
           <t>Saga v2.1→v2.11 (HEAD 8bc7f30). 3 capas defensivas: HTML head script inline (CSS lock + flag + skip splash), main-entry guard, ui-nav showPage lock-aware. Plus: auth.js INITIAL_SESSION-only restore.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="38" t="inlineStr">
+        <is>
+          <t>ERR-24</t>
+        </is>
+      </c>
+      <c r="B27" s="38" t="inlineStr">
+        <is>
+          <t>Wikipedia sin cobertura masiva de páginas "[País]_national_football_team_all-time_record"</t>
+        </is>
+      </c>
+      <c r="C27" s="38" t="inlineStr">
+        <is>
+          <t>Solo ~3/48 selecciones tienen esa página. Encabezados y formato wikitext inconsistentes entre las que sí existen.</t>
+        </is>
+      </c>
+      <c r="D27" s="38" t="inlineStr">
+        <is>
+          <t>Migrar a 11v11.com/stats (Fase D.2 commit bbad657). Validar ≥5 muestras heterogéneas antes de elegir una fuente para scraping masivo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="38" t="inlineStr">
+        <is>
+          <t>ERR-25</t>
+        </is>
+      </c>
+      <c r="B28" s="38" t="inlineStr">
+        <is>
+          <t>fetch a 11v11.com devuelve HTTP 403 sin 3 headers obligatorios</t>
+        </is>
+      </c>
+      <c r="C28" s="38" t="inlineStr">
+        <is>
+          <t>Anti-bot básico: exige User-Agent de Chrome real + Accept: text/html + Accept-Language: en-US. Faltar cualquiera = 403.</t>
+        </is>
+      </c>
+      <c r="D28" s="38" t="inlineStr">
+        <is>
+          <t>Constante fetchHeaders top-level en supabase/functions/porra-ia-compute/index.ts con los 3 headers. Aplicado en handleScrapeH2h y handleScrapeLast5.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="38" t="inlineStr">
+        <is>
+          <t>ERR-26</t>
+        </is>
+      </c>
+      <c r="B29" s="38" t="inlineStr">
+        <is>
+          <t>pg_net no soporta HTTP PUT: no se puede mergear PR desde Supabase</t>
+        </is>
+      </c>
+      <c r="C29" s="38" t="inlineStr">
+        <is>
+          <t>pg_net solo expone net.http_get / net.http_post / net.http_delete. Merge de GitHub requiere PUT /repos/:owner/:repo/pulls/:n/merge.</t>
+        </is>
+      </c>
+      <c r="D29" s="38" t="inlineStr">
+        <is>
+          <t>Workaround: deploy directo del código con deploy_edge_function (evita PUT). PR se mergea después desde MCP GitHub / UI / gh CLI.</t>
         </is>
       </c>
     </row>
@@ -4426,7 +4530,767 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;C&amp;B Esquema Porra Mundial 2026 &amp;R Actualizado: 20 abr 2026 noche (HEAD 8bc7f30)&amp;R Actualizado: 20 abr 2026 (commit 0d3d636)</oddFooter>
+    <oddFooter>&amp;C&amp;B Esquema Porra Mundial 2026 &amp;R Actualizado: 21 abr 2026 (IA Predictor A-C)&amp;R Actualizado: 20 abr 2026 noche (HEAD 8bc7f30)&amp;R Actualizado: 20 abr 2026 (commit 0d3d636)</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D45"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="45" customWidth="1" min="3" max="3"/>
+    <col width="55" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="36" t="inlineStr">
+        <is>
+          <t>PORRA MUNDIAL 2026 — IA Predictor (Fases A-F)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="37" t="inlineStr">
+        <is>
+          <t>Arquitectura 3 capas</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Capa</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Responsable</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Entrada</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Salida</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="35" t="inlineStr">
+        <is>
+          <t>1 — Ingesta</t>
+        </is>
+      </c>
+      <c r="B5" s="35" t="inlineStr">
+        <is>
+          <t>EF porra-ia-compute (4 actions scraper)</t>
+        </is>
+      </c>
+      <c r="C5" s="35" t="inlineStr">
+        <is>
+          <t>Wikipedia Module:SportsRankings (ELO) + 11v11.com (H2H, últimos N)</t>
+        </is>
+      </c>
+      <c r="D5" s="35" t="inlineStr">
+        <is>
+          <t>Tablas ia_elo_fifa, ia_h2h, ia_last5_results</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="35" t="inlineStr">
+        <is>
+          <t>2 — Cómputo</t>
+        </is>
+      </c>
+      <c r="B6" s="35" t="inlineStr">
+        <is>
+          <t>EF porra-ia-compute action=compute (Fase E pendiente)</t>
+        </is>
+      </c>
+      <c r="C6" s="35" t="inlineStr">
+        <is>
+          <t>ia_elo_fifa + ia_h2h + ia_last5_results + partido {home,away}</t>
+        </is>
+      </c>
+      <c r="D6" s="35" t="inlineStr">
+        <is>
+          <t>ia_predictions (sign 1|X|2, confidence 0-100, breakdown JSONB)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="35" t="inlineStr">
+        <is>
+          <t>3 — Consumo</t>
+        </is>
+      </c>
+      <c r="B7" s="35" t="inlineStr">
+        <is>
+          <t>Frontend scoring.js / ko.js (Fase F pendiente)</t>
+        </is>
+      </c>
+      <c r="C7" s="35" t="inlineStr">
+        <is>
+          <t>ia_predictions (RLS public read via policy ia_predictions_public_read)</t>
+        </is>
+      </c>
+      <c r="D7" s="35" t="inlineStr">
+        <is>
+          <t>Tarjeta partido con pronóstico IA + bonus +1 pt si usuario opuesto y acierta</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="37" t="inlineStr">
+        <is>
+          <t>Fórmula del pronóstico (Fase E)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Señal</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Peso</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Peso (fallback sin H2H)</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Notas</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="35" t="inlineStr">
+        <is>
+          <t>ELO FIFA</t>
+        </is>
+      </c>
+      <c r="B11" s="35" t="inlineStr">
+        <is>
+          <t>50%</t>
+        </is>
+      </c>
+      <c r="C11" s="35" t="inlineStr">
+        <is>
+          <t>66%</t>
+        </is>
+      </c>
+      <c r="D11" s="35" t="inlineStr">
+        <is>
+          <t>ia_elo_fifa.elo_points. Fuente: Wikipedia Module:SportsRankings (incluye amistosos).</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="35" t="inlineStr">
+        <is>
+          <t>H2H histórico</t>
+        </is>
+      </c>
+      <c r="B12" s="35" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="C12" s="35" t="inlineStr">
+        <is>
+          <t>0% (fallback)</t>
+        </is>
+      </c>
+      <c r="D12" s="35" t="inlineStr">
+        <is>
+          <t>ia_h2h. Fuente 11v11.com/stats (RSSSF-backed). Si el pair no tiene partido histórico, rebalancear.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="35" t="inlineStr">
+        <is>
+          <t>Racha últimos N</t>
+        </is>
+      </c>
+      <c r="B13" s="35" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="C13" s="35" t="inlineStr">
+        <is>
+          <t>34%</t>
+        </is>
+      </c>
+      <c r="D13" s="35" t="inlineStr">
+        <is>
+          <t>ia_last5_results.results (JSONB). N=8 default, ampliable a N=10 antes del 11 jun vía body.limit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="40" t="inlineStr">
+        <is>
+          <t>Umbrales signo 1|X|2 sobre raw_home_pct: &gt;60% → 1 · 40-60% → X · &lt;40% → 2.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="37" t="inlineStr">
+        <is>
+          <t>Tablas Supabase (migración 20260421_create_ia_predictor_tables.sql, Fase A)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Tabla</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>PK / índices</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Columnas clave</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Origen / RLS</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="35" t="inlineStr">
+        <is>
+          <t>ia_elo_fifa</t>
+        </is>
+      </c>
+      <c r="B18" s="35" t="inlineStr">
+        <is>
+          <t>PK team_code (ISO-3). Index idx_ia_elo_fifa_scraped implícito.</t>
+        </is>
+      </c>
+      <c r="C18" s="35" t="inlineStr">
+        <is>
+          <t>team_code, team_name, elo_points NUMERIC(7,2), rank_position, scraped_at, source</t>
+        </is>
+      </c>
+      <c r="D18" s="35" t="inlineStr">
+        <is>
+          <t>Wikipedia Module:SportsRankings (Fase B.2). RLS enabled, sin policy pública (service role only).</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="35" t="inlineStr">
+        <is>
+          <t>ia_last5_results</t>
+        </is>
+      </c>
+      <c r="B19" s="35" t="inlineStr">
+        <is>
+          <t>PK team_code (FK → ia_elo_fifa.team_code ON DELETE CASCADE). Index idx_ia_last5_scraped (scraped_at DESC).</t>
+        </is>
+      </c>
+      <c r="C19" s="35" t="inlineStr">
+        <is>
+          <t>team_code, results JSONB (array N objects {date, opponent_name, opponent_iso3, venue, result, gf, ga, competition}), wins, draws, losses, scraped_at</t>
+        </is>
+      </c>
+      <c r="D19" s="35" t="inlineStr">
+        <is>
+          <t>11v11.com/teams/{slug}/tab/matches/ (Fase C). RLS enabled, sin policy pública.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="35" t="inlineStr">
+        <is>
+          <t>ia_h2h</t>
+        </is>
+      </c>
+      <c r="B20" s="35" t="inlineStr">
+        <is>
+          <t>PK (team_a_code, team_b_code) con CHECK h2h_alphabetical (team_a &lt; team_b).</t>
+        </is>
+      </c>
+      <c r="C20" s="35" t="inlineStr">
+        <is>
+          <t>team_a_code, team_b_code, matches JSONB {total, gf_team_a, ga_team_a, source_team, source}, team_a_wins, team_b_wins, draws, last_played (DATE, null en 11v11 agregado), scraped_at</t>
+        </is>
+      </c>
+      <c r="D20" s="35" t="inlineStr">
+        <is>
+          <t>11v11.com/teams/{slug}/tab/stats/ (Fase D.2). RLS enabled, sin policy pública. Dedup por pair antes de UPSERT (ON CONFLICT no admite misma fila 2x).</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="35" t="inlineStr">
+        <is>
+          <t>ia_predictions</t>
+        </is>
+      </c>
+      <c r="B21" s="35" t="inlineStr">
+        <is>
+          <t>PK match_id. Index idx_ia_predictions_computed (computed_at DESC).</t>
+        </is>
+      </c>
+      <c r="C21" s="35" t="inlineStr">
+        <is>
+          <t>match_id, home_code, away_code, sign CHAR(1) CHECK (1|X|2), confidence SMALLINT 0-100, breakdown JSONB {elo_score, h2h_score, last5_score, raw_home_pct}, used_fallback BOOLEAN, computed_at</t>
+        </is>
+      </c>
+      <c r="D21" s="35" t="inlineStr">
+        <is>
+          <t>EF compute (Fase E pendiente). **RLS + policy ia_predictions_public_read**: cualquier authenticated SELECT. Lectura desde frontend.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="37" t="inlineStr">
+        <is>
+          <t>Estado Fases A-F (21 abr 2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>Fase</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Acción / Entregable</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>Commit / PR</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>Estado</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="35" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B25" s="35" t="inlineStr">
+        <is>
+          <t>Migración 4 tablas ia_* + EF porra-ia-compute esqueleto (router status/scrape_elo/scrape_last5/scrape_h2h/compute)</t>
+        </is>
+      </c>
+      <c r="C25" s="35" t="inlineStr">
+        <is>
+          <t>968332a (PR #10)</t>
+        </is>
+      </c>
+      <c r="D25" s="35" t="inlineStr">
+        <is>
+          <t>✅ Merged + migración aplicada</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="41" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="B26" s="41" t="inlineStr">
+        <is>
+          <t>scrape_elo via inside.fifa.com/api/ranking-overview</t>
+        </is>
+      </c>
+      <c r="C26" s="41" t="inlineStr">
+        <is>
+          <t>4a32737 (PR #11)</t>
+        </is>
+      </c>
+      <c r="D26" s="41" t="inlineStr">
+        <is>
+          <t>⚠️ Deprecada: solo datos hasta sept 2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="35" t="inlineStr">
+        <is>
+          <t>B.2</t>
+        </is>
+      </c>
+      <c r="B27" s="35" t="inlineStr">
+        <is>
+          <t>scrape_elo via Wikipedia Module:SportsRankings/data/FIFA_World_Rankings (MediaWiki API + regex Lua)</t>
+        </is>
+      </c>
+      <c r="C27" s="35" t="inlineStr">
+        <is>
+          <t>c845f3e (PR #12)</t>
+        </is>
+      </c>
+      <c r="D27" s="35" t="inlineStr">
+        <is>
+          <t>✅ Merged + desplegada (v3). 211 países upserted.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="41" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="B28" s="41" t="inlineStr">
+        <is>
+          <t>scrape_h2h via Wikipedia [País]_national_football_team_all-time_record</t>
+        </is>
+      </c>
+      <c r="C28" s="41" t="inlineStr">
+        <is>
+          <t>cba5dcc (PR #13)</t>
+        </is>
+      </c>
+      <c r="D28" s="41" t="inlineStr">
+        <is>
+          <t>⚠️ Deprecada: solo ~3/48 tienen página (ERR-24)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="35" t="inlineStr">
+        <is>
+          <t>D.2</t>
+        </is>
+      </c>
+      <c r="B29" s="35" t="inlineStr">
+        <is>
+          <t>scrape_h2h via 11v11.com/teams/{slug}/tab/stats/ (HTML regex, headers Chrome obligatorios)</t>
+        </is>
+      </c>
+      <c r="C29" s="35" t="inlineStr">
+        <is>
+          <t>bbad657 (PR #14)</t>
+        </is>
+      </c>
+      <c r="D29" s="35" t="inlineStr">
+        <is>
+          <t>✅ Merged + desplegada (v5). 815 pairs upserted (72% cobertura).</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="39" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="B30" s="39" t="inlineStr">
+        <is>
+          <t>scrape_last_n via 11v11.com/teams/{slug}/tab/matches/ (default N=8, limit parametrizable 1-20)</t>
+        </is>
+      </c>
+      <c r="C30" s="39" t="inlineStr">
+        <is>
+          <t>5a87f1e (rama claude/fase-c-last-n, PR #15)</t>
+        </is>
+      </c>
+      <c r="D30" s="39" t="inlineStr">
+        <is>
+          <t>🟡 EF v6 desplegada desde rama. PR abierto pendiente de merge (ERR-26).</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="35" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="B31" s="35" t="inlineStr">
+        <is>
+          <t>handleCompute: leer ELO + H2H + Racha, aplicar fórmula 50/25/25 con fallback 66/34, UPSERT ia_predictions</t>
+        </is>
+      </c>
+      <c r="C31" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D31" s="35" t="inlineStr">
+        <is>
+          <t>⏳ Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="35" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="B32" s="35" t="inlineStr">
+        <is>
+          <t>Frontend scoring.js / ko.js: leer ia_predictions, pintar pronóstico en tarjeta, calcular bonus +1 IA-opuesta</t>
+        </is>
+      </c>
+      <c r="C32" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D32" s="35" t="inlineStr">
+        <is>
+          <t>⏳ Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="37" t="inlineStr">
+        <is>
+          <t>Estado tablas al 21 abr PM</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>Tabla</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>Filas</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>Última ingesta</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>Notas</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="35" t="inlineStr">
+        <is>
+          <t>ia_elo_fifa</t>
+        </is>
+      </c>
+      <c r="B36" s="35" t="inlineStr">
+        <is>
+          <t>211</t>
+        </is>
+      </c>
+      <c r="C36" s="35" t="inlineStr">
+        <is>
+          <t>Wikipedia update 2026-04-01</t>
+        </is>
+      </c>
+      <c r="D36" s="35" t="inlineStr">
+        <is>
+          <t>Próximo refresh FIFA 9 jun 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="35" t="inlineStr">
+        <is>
+          <t>ia_h2h</t>
+        </is>
+      </c>
+      <c r="B37" s="35" t="inlineStr">
+        <is>
+          <t>815</t>
+        </is>
+      </c>
+      <c r="C37" s="35" t="inlineStr">
+        <is>
+          <t>21 abr 2026 (Fase D.2 smoke test)</t>
+        </is>
+      </c>
+      <c r="D37" s="35" t="inlineStr">
+        <is>
+          <t>Pares únicos entre mundialistas. 72% de 1.128 teóricos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="35" t="inlineStr">
+        <is>
+          <t>ia_last5_results</t>
+        </is>
+      </c>
+      <c r="B38" s="35" t="inlineStr">
+        <is>
+          <t>48</t>
+        </is>
+      </c>
+      <c r="C38" s="35" t="inlineStr">
+        <is>
+          <t>21 abr 2026 (Fase C smoke test)</t>
+        </is>
+      </c>
+      <c r="D38" s="35" t="inlineStr">
+        <is>
+          <t>N=8 por selección; ARG 7 por caché 11v11. Total ~382 partidos en JSONB.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="35" t="inlineStr">
+        <is>
+          <t>ia_predictions</t>
+        </is>
+      </c>
+      <c r="B39" s="35" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C39" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D39" s="35" t="inlineStr">
+        <is>
+          <t>Poblada por Fase E pendiente.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="37" t="inlineStr">
+        <is>
+          <t>Headers obligatorios 11v11.com (sin los 3 → 403, ver ERR-25)</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>Header</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>Valor</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>Rol</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="35" t="inlineStr">
+        <is>
+          <t>User-Agent</t>
+        </is>
+      </c>
+      <c r="B43" s="35" t="inlineStr">
+        <is>
+          <t>Mozilla/5.0 (Windows NT 10.0; Win64; x64) AppleWebKit/537.36 (KHTML, like Gecko) Chrome/120.0 Safari/537.36</t>
+        </is>
+      </c>
+      <c r="C43" s="35" t="inlineStr">
+        <is>
+          <t>Chrome real. UA custom (ej. pm26-ia-predictor/1.0) devuelve 403.</t>
+        </is>
+      </c>
+      <c r="D43" s="35" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="35" t="inlineStr">
+        <is>
+          <t>Accept</t>
+        </is>
+      </c>
+      <c r="B44" s="35" t="inlineStr">
+        <is>
+          <t>text/html,application/xhtml+xml</t>
+        </is>
+      </c>
+      <c r="C44" s="35" t="inlineStr">
+        <is>
+          <t>Explicita que esperamos HTML</t>
+        </is>
+      </c>
+      <c r="D44" s="35" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="35" t="inlineStr">
+        <is>
+          <t>Accept-Language</t>
+        </is>
+      </c>
+      <c r="B45" s="35" t="inlineStr">
+        <is>
+          <t>en-US,en;q=0.9</t>
+        </is>
+      </c>
+      <c r="C45" s="35" t="inlineStr">
+        <is>
+          <t>Evita redirecciones de i18n del site</t>
+        </is>
+      </c>
+      <c r="D45" s="35" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <mergeCells count="8">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A23:D23"/>
+    <mergeCell ref="A9:D9"/>
+    <mergeCell ref="A34:D34"/>
+    <mergeCell ref="A3:D3"/>
+    <mergeCell ref="A41:D41"/>
+    <mergeCell ref="A16:D16"/>
+    <mergeCell ref="A14:D14"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter>
+    <oddHeader/>
+    <oddFooter>&amp;C&amp;B Esquema Porra Mundial 2026 &amp;R Actualizado: 21 abr 2026 (IA Predictor A-C)</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>

</xml_diff>

<commit_message>
docs(ia-predictor): fix versiones EF (match-live v16, webshare 1.0.7) + bug apify-webhook pending v8 + PR #15 como deuda técnica menor
</commit_message>
<xml_diff>
--- a/ESQUEMA_SISTEMA_PORRA2026.xlsx
+++ b/ESQUEMA_SISTEMA_PORRA2026.xlsx
@@ -753,7 +753,7 @@
     <row r="3" ht="55" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>porra-match-live v13</t>
+          <t>porra-match-live v16</t>
         </is>
       </c>
       <c r="B3" s="4" t="inlineStr">
@@ -795,7 +795,7 @@
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>Procesa resultado del actor. Lee dataset Apify. extractMatchState() desde item.event.data.event + item.incidents.data.incidents. Detecta cambios estado y goles nuevos. Envía WhatsApp. Upsert DB.</t>
+          <t>Procesa resultado del actor. Lee dataset Apify. extractMatchState() desde item.event.data.event + item.incidents.data.incidents. Detecta cambios estado y goles nuevos. Envía WhatsApp. Upsert DB. Bug conocido (pending v8): no persiste home_team_name/away_team_name/competition/match_start_ts.</t>
         </is>
       </c>
       <c r="E4" s="5" t="inlineStr">
@@ -1108,7 +1108,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;C&amp;B Esquema Porra Mundial 2026 &amp;R Actualizado: 21 abr 2026 (IA Predictor A-C)&amp;R Actualizado: 20 abr 2026 noche (HEAD 8bc7f30)&amp;R Actualizado: 20 abr 2026 (commit 0d3d636)</oddFooter>
+    <oddFooter>&amp;C&amp;B Esquema Porra Mundial 2026 &amp;R Actualizado: 21 abr 2026 (IA Predictor A-C)&amp;R Actualizado: 21 abr 2026 (IA Predictor A-C)&amp;R Actualizado: 20 abr 2026 noche (HEAD 8bc7f30)&amp;R Actualizado: 20 abr 2026 (commit 0d3d636)</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -1423,7 +1423,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;C&amp;B Esquema Porra Mundial 2026 &amp;R Actualizado: 21 abr 2026 (IA Predictor A-C)&amp;R Actualizado: 20 abr 2026 noche (HEAD 8bc7f30)&amp;R Actualizado: 20 abr 2026 (commit 0d3d636)</oddFooter>
+    <oddFooter>&amp;C&amp;B Esquema Porra Mundial 2026 &amp;R Actualizado: 21 abr 2026 (IA Predictor A-C)&amp;R Actualizado: 21 abr 2026 (IA Predictor A-C)&amp;R Actualizado: 20 abr 2026 noche (HEAD 8bc7f30)&amp;R Actualizado: 20 abr 2026 (commit 0d3d636)</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -2034,7 +2034,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;C&amp;B Esquema Porra Mundial 2026 &amp;R Actualizado: 21 abr 2026 (IA Predictor A-C)&amp;R Actualizado: 20 abr 2026 noche (HEAD 8bc7f30)&amp;R Actualizado: 20 abr 2026 (commit 0d3d636)</oddFooter>
+    <oddFooter>&amp;C&amp;B Esquema Porra Mundial 2026 &amp;R Actualizado: 21 abr 2026 (IA Predictor A-C)&amp;R Actualizado: 21 abr 2026 (IA Predictor A-C)&amp;R Actualizado: 20 abr 2026 noche (HEAD 8bc7f30)&amp;R Actualizado: 20 abr 2026 (commit 0d3d636)</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -2532,7 +2532,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;C&amp;B Esquema Porra Mundial 2026 &amp;R Actualizado: 21 abr 2026 (IA Predictor A-C)&amp;R Actualizado: 20 abr 2026 noche (HEAD 8bc7f30)&amp;R Actualizado: 20 abr 2026 (commit 0d3d636)</oddFooter>
+    <oddFooter>&amp;C&amp;B Esquema Porra Mundial 2026 &amp;R Actualizado: 21 abr 2026 (IA Predictor A-C)&amp;R Actualizado: 21 abr 2026 (IA Predictor A-C)&amp;R Actualizado: 20 abr 2026 noche (HEAD 8bc7f30)&amp;R Actualizado: 20 abr 2026 (commit 0d3d636)</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -2925,7 +2925,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;C&amp;B Esquema Porra Mundial 2026 &amp;R Actualizado: 21 abr 2026 (IA Predictor A-C)&amp;R Actualizado: 20 abr 2026 noche (HEAD 8bc7f30)&amp;R Actualizado: 20 abr 2026 (commit 0d3d636)</oddFooter>
+    <oddFooter>&amp;C&amp;B Esquema Porra Mundial 2026 &amp;R Actualizado: 21 abr 2026 (IA Predictor A-C)&amp;R Actualizado: 21 abr 2026 (IA Predictor A-C)&amp;R Actualizado: 20 abr 2026 noche (HEAD 8bc7f30)&amp;R Actualizado: 20 abr 2026 (commit 0d3d636)</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -3897,7 +3897,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;C&amp;B Esquema Porra Mundial 2026 &amp;R Actualizado: 21 abr 2026 (IA Predictor A-C)&amp;R Actualizado: 20 abr 2026 noche (HEAD 8bc7f30)&amp;R Actualizado: 20 abr 2026 (commit 0d3d636)</oddFooter>
+    <oddFooter>&amp;C&amp;B Esquema Porra Mundial 2026 &amp;R Actualizado: 21 abr 2026 (IA Predictor A-C)&amp;R Actualizado: 21 abr 2026 (IA Predictor A-C)&amp;R Actualizado: 20 abr 2026 noche (HEAD 8bc7f30)&amp;R Actualizado: 20 abr 2026 (commit 0d3d636)</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -4530,7 +4530,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;C&amp;B Esquema Porra Mundial 2026 &amp;R Actualizado: 21 abr 2026 (IA Predictor A-C)&amp;R Actualizado: 20 abr 2026 noche (HEAD 8bc7f30)&amp;R Actualizado: 20 abr 2026 (commit 0d3d636)</oddFooter>
+    <oddFooter>&amp;C&amp;B Esquema Porra Mundial 2026 &amp;R Actualizado: 21 abr 2026 (IA Predictor A-C)&amp;R Actualizado: 21 abr 2026 (IA Predictor A-C)&amp;R Actualizado: 20 abr 2026 noche (HEAD 8bc7f30)&amp;R Actualizado: 20 abr 2026 (commit 0d3d636)</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>

</xml_diff>

<commit_message>
docs(ia-predictor): checkpoint cierre Fase E — EF v9 ACTIVE, paridad 46/46, ERR-27
</commit_message>
<xml_diff>
--- a/ESQUEMA_SISTEMA_PORRA2026.xlsx
+++ b/ESQUEMA_SISTEMA_PORRA2026.xlsx
@@ -13,7 +13,7 @@
     <sheet name="Flujo + Leyenda" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="IDs SofaScore + Costes" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Frontend Mobile" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Errores ERR-01..ERR-26" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Errores ERR-01..ERR-27" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="IA Predictor" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
@@ -1077,7 +1077,7 @@
     <row r="15">
       <c r="A15" s="38" t="inlineStr">
         <is>
-          <t>porra-ia-compute v6</t>
+          <t>porra-ia-compute v9</t>
         </is>
       </c>
       <c r="B15" s="38" t="inlineStr">
@@ -1092,12 +1092,12 @@
       </c>
       <c r="D15" s="38" t="inlineStr">
         <is>
-          <t>IA Predictor (Fases A-C implementadas). Router: status / scrape_elo (Wikipedia Module:SportsRankings → ia_elo_fifa) / scrape_h2h (11v11.com/stats → ia_h2h) / scrape_last5 (11v11.com/matches → ia_last5_results) / compute (Fase E pendiente). verify_jwt=false.</t>
+          <t>IA Predictor (Fases A-E cerradas). 7 actions: status / scrape_elo (Wikipedia Module) / scrape_h2h (11v11.com/stats) / scrape_last5 (11v11.com/matches) / freeze_snapshot (scrapes + crea snapshot + activa) / compute_groups (72 partidos grupos) / compute_match (on-demand KO, rate limit 30/min). Motor log-odds+softmax pesos 75/10/15 (fallback 85/0/15), home adv +85/+95 MEX. Quip Haiku. verify_jwt=false. Paridad Python↔TS 46/46.</t>
         </is>
       </c>
       <c r="E15" s="38" t="inlineStr">
         <is>
-          <t>✅ En producción (Fases A-C). Fase E/F pendientes.</t>
+          <t>✅ En producción v9 (paridad verde, smoke tests OK)</t>
         </is>
       </c>
     </row>
@@ -1108,7 +1108,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;C&amp;B Esquema Porra Mundial 2026 &amp;R Actualizado: 21 abr 2026 (IA Predictor A-C)&amp;R Actualizado: 21 abr 2026 (IA Predictor A-C)&amp;R Actualizado: 20 abr 2026 noche (HEAD 8bc7f30)&amp;R Actualizado: 20 abr 2026 (commit 0d3d636)</oddFooter>
+    <oddFooter>&amp;C&amp;B Esquema Porra Mundial 2026 &amp;R Actualizado: 21 abr 2026 noche (Fase E cerrada — EF v9)&amp;R Actualizado: 21 abr 2026 (IA Predictor A-C)&amp;R Actualizado: 21 abr 2026 (IA Predictor A-C)&amp;R Actualizado: 20 abr 2026 noche (HEAD 8bc7f30)&amp;R Actualizado: 20 abr 2026 (commit 0d3d636)</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -1423,7 +1423,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;C&amp;B Esquema Porra Mundial 2026 &amp;R Actualizado: 21 abr 2026 (IA Predictor A-C)&amp;R Actualizado: 21 abr 2026 (IA Predictor A-C)&amp;R Actualizado: 20 abr 2026 noche (HEAD 8bc7f30)&amp;R Actualizado: 20 abr 2026 (commit 0d3d636)</oddFooter>
+    <oddFooter>&amp;C&amp;B Esquema Porra Mundial 2026 &amp;R Actualizado: 21 abr 2026 noche (Fase E cerrada — EF v9)&amp;R Actualizado: 21 abr 2026 (IA Predictor A-C)&amp;R Actualizado: 21 abr 2026 (IA Predictor A-C)&amp;R Actualizado: 20 abr 2026 noche (HEAD 8bc7f30)&amp;R Actualizado: 20 abr 2026 (commit 0d3d636)</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -2034,7 +2034,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;C&amp;B Esquema Porra Mundial 2026 &amp;R Actualizado: 21 abr 2026 (IA Predictor A-C)&amp;R Actualizado: 21 abr 2026 (IA Predictor A-C)&amp;R Actualizado: 20 abr 2026 noche (HEAD 8bc7f30)&amp;R Actualizado: 20 abr 2026 (commit 0d3d636)</oddFooter>
+    <oddFooter>&amp;C&amp;B Esquema Porra Mundial 2026 &amp;R Actualizado: 21 abr 2026 noche (Fase E cerrada — EF v9)&amp;R Actualizado: 21 abr 2026 (IA Predictor A-C)&amp;R Actualizado: 21 abr 2026 (IA Predictor A-C)&amp;R Actualizado: 20 abr 2026 noche (HEAD 8bc7f30)&amp;R Actualizado: 20 abr 2026 (commit 0d3d636)</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -2532,7 +2532,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;C&amp;B Esquema Porra Mundial 2026 &amp;R Actualizado: 21 abr 2026 (IA Predictor A-C)&amp;R Actualizado: 21 abr 2026 (IA Predictor A-C)&amp;R Actualizado: 20 abr 2026 noche (HEAD 8bc7f30)&amp;R Actualizado: 20 abr 2026 (commit 0d3d636)</oddFooter>
+    <oddFooter>&amp;C&amp;B Esquema Porra Mundial 2026 &amp;R Actualizado: 21 abr 2026 noche (Fase E cerrada — EF v9)&amp;R Actualizado: 21 abr 2026 (IA Predictor A-C)&amp;R Actualizado: 21 abr 2026 (IA Predictor A-C)&amp;R Actualizado: 20 abr 2026 noche (HEAD 8bc7f30)&amp;R Actualizado: 20 abr 2026 (commit 0d3d636)</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -2925,7 +2925,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;C&amp;B Esquema Porra Mundial 2026 &amp;R Actualizado: 21 abr 2026 (IA Predictor A-C)&amp;R Actualizado: 21 abr 2026 (IA Predictor A-C)&amp;R Actualizado: 20 abr 2026 noche (HEAD 8bc7f30)&amp;R Actualizado: 20 abr 2026 (commit 0d3d636)</oddFooter>
+    <oddFooter>&amp;C&amp;B Esquema Porra Mundial 2026 &amp;R Actualizado: 21 abr 2026 noche (Fase E cerrada — EF v9)&amp;R Actualizado: 21 abr 2026 (IA Predictor A-C)&amp;R Actualizado: 21 abr 2026 (IA Predictor A-C)&amp;R Actualizado: 20 abr 2026 noche (HEAD 8bc7f30)&amp;R Actualizado: 20 abr 2026 (commit 0d3d636)</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -3897,7 +3897,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;C&amp;B Esquema Porra Mundial 2026 &amp;R Actualizado: 21 abr 2026 (IA Predictor A-C)&amp;R Actualizado: 21 abr 2026 (IA Predictor A-C)&amp;R Actualizado: 20 abr 2026 noche (HEAD 8bc7f30)&amp;R Actualizado: 20 abr 2026 (commit 0d3d636)</oddFooter>
+    <oddFooter>&amp;C&amp;B Esquema Porra Mundial 2026 &amp;R Actualizado: 21 abr 2026 noche (Fase E cerrada — EF v9)&amp;R Actualizado: 21 abr 2026 (IA Predictor A-C)&amp;R Actualizado: 21 abr 2026 (IA Predictor A-C)&amp;R Actualizado: 20 abr 2026 noche (HEAD 8bc7f30)&amp;R Actualizado: 20 abr 2026 (commit 0d3d636)</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -3912,7 +3912,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D29"/>
+  <dimension ref="A1:D30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -3928,7 +3928,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -4520,6 +4519,28 @@
       <c r="D29" s="38" t="inlineStr">
         <is>
           <t>Workaround: deploy directo del código con deploy_edge_function (evita PUT). PR se mergea después desde MCP GitHub / UI / gh CLI.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="38" t="inlineStr">
+        <is>
+          <t>ERR-27</t>
+        </is>
+      </c>
+      <c r="B30" s="38" t="inlineStr">
+        <is>
+          <t>supa.from("vault.decrypted_secrets") / .schema("vault") → readVaultSecret devuelve null silenciosamente → 401 en freeze_snapshot</t>
+        </is>
+      </c>
+      <c r="C30" s="38" t="inlineStr">
+        <is>
+          <t>PostgREST interpreta "vault.decrypted_secrets" como nombre literal de tabla en schema public. .schema("vault") tampoco funciona porque el schema vault NO está expuesto en api.schemas del proyecto.</t>
+        </is>
+      </c>
+      <c r="D30" s="38" t="inlineStr">
+        <is>
+          <t>Fix: RPC get_vault_secrets(secret_names text[]) vía fetch directo a /rest/v1/rpc/... con apikey + Authorization Bearer = SUPABASE_SERVICE_ROLE_KEY. Mismo patrón probado en porra-fix-encoding v6. Commit a210598.</t>
         </is>
       </c>
     </row>
@@ -4530,7 +4551,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;C&amp;B Esquema Porra Mundial 2026 &amp;R Actualizado: 21 abr 2026 (IA Predictor A-C)&amp;R Actualizado: 21 abr 2026 (IA Predictor A-C)&amp;R Actualizado: 20 abr 2026 noche (HEAD 8bc7f30)&amp;R Actualizado: 20 abr 2026 (commit 0d3d636)</oddFooter>
+    <oddFooter>&amp;C&amp;B Esquema Porra Mundial 2026 &amp;R Actualizado: 21 abr 2026 noche (Fase E cerrada — EF v9)&amp;R Actualizado: 21 abr 2026 (IA Predictor A-C)&amp;R Actualizado: 21 abr 2026 (IA Predictor A-C)&amp;R Actualizado: 20 abr 2026 noche (HEAD 8bc7f30)&amp;R Actualizado: 20 abr 2026 (commit 0d3d636)</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -4861,17 +4882,17 @@
       </c>
       <c r="B21" s="35" t="inlineStr">
         <is>
-          <t>PK match_id. Index idx_ia_predictions_computed (computed_at DESC).</t>
+          <t>PK match_id. FK snapshot_id → ia_snapshots(id). Index idx_ia_predictions_lookup (home_code, away_code, snapshot_id).</t>
         </is>
       </c>
       <c r="C21" s="35" t="inlineStr">
         <is>
-          <t>match_id, home_code, away_code, sign CHAR(1) CHECK (1|X|2), confidence SMALLINT 0-100, breakdown JSONB {elo_score, h2h_score, last5_score, raw_home_pct}, used_fallback BOOLEAN, computed_at</t>
+          <t>match_id, home_code, away_code, sign CHAR(1) CHECK (1|X|2), confidence SMALLINT 0-100, breakdown JSONB {elo_signal, h2h_signal, racha_signal, draw_score, home_advantage, weights_used, scores, p_*, p_max, margin, is_dudoso, quip}, used_fallback BOOLEAN, is_ko_ondemand BOOLEAN, snapshot_id BIGINT, computed_at</t>
         </is>
       </c>
       <c r="D21" s="35" t="inlineStr">
         <is>
-          <t>EF compute (Fase E pendiente). **RLS + policy ia_predictions_public_read**: cualquier authenticated SELECT. Lectura desde frontend.</t>
+          <t>EF compute_groups / compute_match (Fase E). RLS + policy ia_predictions_public_read: authenticated SELECT (frontend consumirá desde scoring.js / ko.js en Fase F).</t>
         </is>
       </c>
     </row>
@@ -5027,12 +5048,12 @@
       </c>
       <c r="C30" s="39" t="inlineStr">
         <is>
-          <t>5a87f1e (rama claude/fase-c-last-n, PR #15)</t>
-        </is>
-      </c>
-      <c r="D30" s="39" t="inlineStr">
-        <is>
-          <t>🟡 EF v6 desplegada desde rama. PR abierto pendiente de merge (ERR-26).</t>
+          <t>2904025 (squash-merge de PR #15)</t>
+        </is>
+      </c>
+      <c r="D30" s="38" t="inlineStr">
+        <is>
+          <t>✅ Merged + desplegada (EF v6 original; ahora v9)</t>
         </is>
       </c>
     </row>
@@ -5044,17 +5065,17 @@
       </c>
       <c r="B31" s="35" t="inlineStr">
         <is>
-          <t>handleCompute: leer ELO + H2H + Racha, aplicar fórmula 50/25/25 con fallback 66/34, UPSERT ia_predictions</t>
+          <t>Motor IA log-odds+softmax portado desde predictor.py. 3 actions nuevas: freeze_snapshot (scrapes serie + crea snapshot + activa + WhatsApp), compute_groups (72 partidos grupos, quip concurrency 5), compute_match (on-demand KO + cache BD + rate limit 30/min). Pesos 75/10/15 (fallback 85/0/15). Home adv +85/+95 MEX. Margen dudoso 0.08. Quip Haiku 4.5. ia_snapshots con invariante "1 activo". Cron 11 jun 00:00 UTC freeze + 00:10 groups.</t>
         </is>
       </c>
       <c r="C31" s="35" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D31" s="35" t="inlineStr">
-        <is>
-          <t>⏳ Pendiente</t>
+          <t>8d8b667 (PR #16)</t>
+        </is>
+      </c>
+      <c r="D31" s="38" t="inlineStr">
+        <is>
+          <t>✅ Merged + desplegada (EF v9). Paridad Python↔TS 46/46 verde. Smoke tests OK.</t>
         </is>
       </c>
     </row>
@@ -5080,10 +5101,11 @@
         </is>
       </c>
     </row>
+    <row r="33"/>
     <row r="34">
       <c r="A34" s="37" t="inlineStr">
         <is>
-          <t>Estado tablas al 21 abr PM</t>
+          <t>Estado tablas al 21 abr 2026 (noche, tras cierre Fase E)</t>
         </is>
       </c>
     </row>
@@ -5183,17 +5205,39 @@
       </c>
       <c r="B39" s="35" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>on-demand (crece en runtime)</t>
         </is>
       </c>
       <c r="C39" s="35" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>21 abr 2026 noche (smoke test compute_match)</t>
         </is>
       </c>
       <c r="D39" s="35" t="inlineStr">
         <is>
-          <t>Poblada por Fase E pendiente.</t>
+          <t>Poblada vía compute_match on-demand. Batch de 72 filas de fase de grupos prevista del cron ia-compute-groups-mundial el 11 jun 00:10 UTC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="38" t="inlineStr">
+        <is>
+          <t>ia_snapshots</t>
+        </is>
+      </c>
+      <c r="B40" s="38" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C40" s="38" t="inlineStr">
+        <is>
+          <t>21 abr 2026 noche (smoke test + productivo)</t>
+        </is>
+      </c>
+      <c r="D40" s="38" t="inlineStr">
+        <is>
+          <t>Snapshot activo: id=2 label="initial_test_21apr". Invariante "1 activo" reforzado por unique index parcial. Cleanup nocturno de inactivos &gt;7d.</t>
         </is>
       </c>
     </row>
@@ -5290,7 +5334,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;C&amp;B Esquema Porra Mundial 2026 &amp;R Actualizado: 21 abr 2026 (IA Predictor A-C)</oddFooter>
+    <oddFooter>&amp;C&amp;B Esquema Porra Mundial 2026 &amp;R Actualizado: 21 abr 2026 noche (Fase E cerrada — EF v9)&amp;R Actualizado: 21 abr 2026 (IA Predictor A-C)</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>

</xml_diff>